<commit_message>
feat: LibreOffice Excel to PDF conversion
- Add ExcelToPdfConverterService using LibreOffice headless
- Auto-generate PDF alongside Excel for AllDocuments and FullDocuments
- Support configurable libreoffice path and timeout via application.yml
- Frontend attachment list shows PDF tags (AllDocumentsPdf/FullDocumentsPdf)
- Dashboard quick menu single row layout with flex
- PDF display name cleanup: remove UUID and redundant prefix
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/alltemple_template-lead.xlsx
+++ b/backend/src/main/resources/templates/alltemple_template-lead.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13380"/>
+    <workbookView windowWidth="29868" windowHeight="13380" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="报关单" sheetId="1" r:id="rId1"/>
@@ -2061,20 +2061,20 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>250825</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>138430</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>480695</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>141605</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>609600</xdr:colOff>
+      <xdr:colOff>739140</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:rowOff>149860</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2" descr="73c7f05700406c30116bf7709ac3f4b7"/>
+        <xdr:cNvPr id="2" name="图片 1" descr="73c7f05700406c30116bf7709ac3f4b7"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -2087,8 +2087,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4040505" y="7342505"/>
-          <a:ext cx="1903095" cy="1652270"/>
+          <a:off x="3747135" y="6979920"/>
+          <a:ext cx="2326005" cy="2019935"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
fix: update invoice templates and supplement service
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/alltemple_template-lead.xlsx
+++ b/backend/src/main/resources/templates/alltemple_template-lead.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13380" activeTab="1"/>
+    <workbookView windowWidth="29868" windowHeight="13380"/>
   </bookViews>
   <sheets>
     <sheet name="报关单" sheetId="1" r:id="rId1"/>
@@ -1549,7 +1549,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1875,6 +1875,54 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="11" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="177" fontId="11" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1882,45 +1930,6 @@
     </xf>
     <xf numFmtId="178" fontId="11" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3016,9 +3025,9 @@
       <c r="E22" s="80"/>
       <c r="F22" s="80"/>
       <c r="G22" s="119"/>
-      <c r="H22" s="120"/>
-      <c r="I22" s="121"/>
-      <c r="J22" s="122"/>
+      <c r="H22" s="136"/>
+      <c r="I22" s="137"/>
+      <c r="J22" s="138"/>
       <c r="K22" s="123"/>
       <c r="L22" s="119"/>
       <c r="M22" s="80"/>
@@ -3070,9 +3079,9 @@
       <c r="E25" s="80"/>
       <c r="F25" s="80"/>
       <c r="G25" s="119"/>
-      <c r="H25" s="121"/>
-      <c r="I25" s="121"/>
-      <c r="J25" s="122"/>
+      <c r="H25" s="137"/>
+      <c r="I25" s="137"/>
+      <c r="J25" s="138"/>
       <c r="K25" s="123"/>
       <c r="L25" s="119"/>
       <c r="M25" s="80"/>
@@ -3117,31 +3126,31 @@
       <c r="R27" s="125"/>
     </row>
     <row r="28" s="71" customFormat="1" ht="16.5" customHeight="1" spans="1:20">
-      <c r="A28" s="136"/>
-      <c r="B28" s="137"/>
-      <c r="C28" s="137"/>
-      <c r="D28" s="138" t="s">
+      <c r="A28" s="139"/>
+      <c r="B28" s="140"/>
+      <c r="C28" s="140"/>
+      <c r="D28" s="141" t="s">
         <v>78</v>
       </c>
-      <c r="E28" s="137"/>
-      <c r="F28" s="137"/>
-      <c r="G28" s="137" t="s">
+      <c r="E28" s="140"/>
+      <c r="F28" s="140"/>
+      <c r="G28" s="140" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="137"/>
-      <c r="I28" s="137"/>
-      <c r="J28" s="138" t="s">
+      <c r="H28" s="140"/>
+      <c r="I28" s="140"/>
+      <c r="J28" s="141" t="s">
         <v>80</v>
       </c>
       <c r="K28" s="116"/>
       <c r="L28" s="116"/>
-      <c r="M28" s="137"/>
-      <c r="N28" s="137"/>
-      <c r="O28" s="138" t="s">
+      <c r="M28" s="140"/>
+      <c r="N28" s="140"/>
+      <c r="O28" s="141" t="s">
         <v>81</v>
       </c>
       <c r="P28" s="116"/>
-      <c r="Q28" s="139"/>
+      <c r="Q28" s="142"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" spans="1:20">
       <c r="A29" s="79" t="s">
@@ -3182,25 +3191,25 @@
       <c r="K30" s="87"/>
       <c r="L30" s="87"/>
       <c r="M30" s="96"/>
-      <c r="Q30" s="140"/>
+      <c r="Q30" s="143"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" spans="1:20">
-      <c r="A31" s="141" t="s">
+      <c r="A31" s="144" t="s">
         <v>85</v>
       </c>
       <c r="B31" s="78"/>
-      <c r="C31" s="142"/>
+      <c r="C31" s="145"/>
       <c r="D31" s="78"/>
       <c r="E31" s="78"/>
       <c r="F31" s="78"/>
       <c r="G31" s="78"/>
-      <c r="H31" s="143"/>
-      <c r="I31" s="143"/>
-      <c r="J31" s="142" t="s">
+      <c r="H31" s="146"/>
+      <c r="I31" s="146"/>
+      <c r="J31" s="145" t="s">
         <v>86</v>
       </c>
       <c r="K31" s="78"/>
-      <c r="L31" s="143"/>
+      <c r="L31" s="146"/>
       <c r="M31" s="102"/>
       <c r="N31" s="78"/>
       <c r="O31" s="78"/>
@@ -3208,7 +3217,7 @@
       <c r="Q31" s="97"/>
     </row>
     <row r="32" ht="16.5" customHeight="1" spans="1:20">
-      <c r="A32" s="144" t="s">
+      <c r="A32" s="147" t="s">
         <v>87</v>
       </c>
       <c r="B32" s="80"/>

</xml_diff>